<commit_message>
se agrego hoja completa y la personalizada
se agrego una funcion para que el programa tenga la opcion de llenar el registro en excel con todos los campos que vienen en el pdf o usar una hoja personalizada por el usuario
</commit_message>
<xml_diff>
--- a/BASE_ALERTAS_NACIONAL_2026_JOAO.bak.xlsx
+++ b/BASE_ALERTAS_NACIONAL_2026_JOAO.bak.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ServicioSocial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF02BB49-800D-410B-A7E0-AA0719046552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B09B7703-1152-4783-90A5-CCA507072CEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="DatosCompletos" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="98">
   <si>
     <t>ID</t>
   </si>
@@ -70,6 +71,39 @@
     <t>AUTORIDAD QUE INGRESO EL REPORTE</t>
   </si>
   <si>
+    <t>¿Habla español?</t>
+  </si>
+  <si>
+    <t>Idioma o lengua indígena</t>
+  </si>
+  <si>
+    <t>Discapacidad</t>
+  </si>
+  <si>
+    <t>Hora de hechos</t>
+  </si>
+  <si>
+    <t>Hora de percato</t>
+  </si>
+  <si>
+    <t>MUNICIPIO</t>
+  </si>
+  <si>
+    <t>Carpeta de investigacion</t>
+  </si>
+  <si>
+    <t>Características físicas</t>
+  </si>
+  <si>
+    <t>Señas particulares</t>
+  </si>
+  <si>
+    <t>Prendas de vestir</t>
+  </si>
+  <si>
+    <t>Lugar de nacimiento</t>
+  </si>
+  <si>
     <t>AN/2846/2026</t>
   </si>
   <si>
@@ -103,55 +137,195 @@
     <t>AN/2847/2026</t>
   </si>
   <si>
+    <t>GILBERTO OSUNA MORALES</t>
+  </si>
+  <si>
+    <t>HOMBRE</t>
+  </si>
+  <si>
+    <t>MASCULINO</t>
+  </si>
+  <si>
+    <t>FI26-10AD9BD19-6E58-4B08-98EA-9E1F5F0437C6</t>
+  </si>
+  <si>
+    <t>SONORA</t>
+  </si>
+  <si>
+    <t>FISCALIA GENERAL DE JUSTICIA DEL ESTADO DE SONORA</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>SIN DATO</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>17:00</t>
+  </si>
+  <si>
+    <t>21:52</t>
+  </si>
+  <si>
+    <t>HERMOSILLO</t>
+  </si>
+  <si>
+    <t>CI/HER/022/06/00156/3-2026</t>
+  </si>
+  <si>
+    <t>CICTARIZ EN EL LABIO INFERIOR</t>
+  </si>
+  <si>
+    <t>AN/2848/2026</t>
+  </si>
+  <si>
+    <t>VICTOR MILLAN BECERRA</t>
+  </si>
+  <si>
+    <t>FI26-112AB3067-BDFC-4E9D-AEDF-39CE4DAADCC6</t>
+  </si>
+  <si>
+    <t>PUEBLA</t>
+  </si>
+  <si>
+    <t>COMISION DE BUSQUEDA DE PERSONAS DEL ESTADO DE PUEBLA</t>
+  </si>
+  <si>
+    <t>02:30</t>
+  </si>
+  <si>
+    <t>JUAN C BONILLA</t>
+  </si>
+  <si>
+    <t>CBP-283/2026</t>
+  </si>
+  <si>
+    <t>COMPLEXION: DELGADACARA: REDONDOCOLOR DE LA PIEL: MORENOCABELLO: NEGRO CORTO LISOOJOS: CAFÉS MEDIANOSNARIZ: NO RECUERDABOCA: MEDIANALABIOS: DELGADOSESTATURA: 178 CM</t>
+  </si>
+  <si>
+    <t>NINGUNA</t>
+  </si>
+  <si>
+    <t>AN/2849/2026</t>
+  </si>
+  <si>
+    <t>CALEB EMMANUEL LAGUNAS ESPINOZA</t>
+  </si>
+  <si>
+    <t>FI26-1C22E33CF-C5E1-4850-AB89-71C5A3210774</t>
+  </si>
+  <si>
+    <t>07:00</t>
+  </si>
+  <si>
+    <t>08:00</t>
+  </si>
+  <si>
+    <t>TLACOTEPEC DE BENITO JUAREZ</t>
+  </si>
+  <si>
+    <t>CBP-285/2026</t>
+  </si>
+  <si>
+    <t>COMPLEXION: DELGADACARA: OVALADOCOLOR DE LA PIEL: MORENOCABELLO: NEGRO CORTO LISOOJOS: CAFÉS MEDIANOSNARIZ: RECTABOCA: PEQUEÑALABIOS: DELGADOSESTATURA: 120 CMPESO: 35KG</t>
+  </si>
+  <si>
+    <t>CUATRO CICATRICES ARRIBA DE LA OREJA EN LA PARTE DERECHA</t>
+  </si>
+  <si>
+    <t>AN/2850/2026</t>
+  </si>
+  <si>
+    <t>AN/2851/2026</t>
+  </si>
+  <si>
+    <t>AN/2852/2026</t>
+  </si>
+  <si>
+    <t>AN/2853/2026</t>
+  </si>
+  <si>
+    <t>AN/2854/2026</t>
+  </si>
+  <si>
+    <t>AN/2855/2026</t>
+  </si>
+  <si>
+    <t>AN/2856/2026</t>
+  </si>
+  <si>
+    <t>AN/2857/2026</t>
+  </si>
+  <si>
+    <t>AN/2858/2026</t>
+  </si>
+  <si>
+    <t>AN/2859/2026</t>
+  </si>
+  <si>
+    <t>AN/2860/2026</t>
+  </si>
+  <si>
+    <t>AN/2961/2026</t>
+  </si>
+  <si>
+    <t>17-06-26</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
     <t>FISCALÍA GENERAL DE JUSTICIA DE LA CIUDAD DE MÉXICO.</t>
   </si>
   <si>
-    <t>AN/2848/2026</t>
-  </si>
-  <si>
-    <t>AN/2849/2026</t>
-  </si>
-  <si>
-    <t>AN/2850/2026</t>
-  </si>
-  <si>
-    <t>AN/2851/2026</t>
-  </si>
-  <si>
-    <t>AN/2852/2026</t>
-  </si>
-  <si>
-    <t>AN/2853/2026</t>
-  </si>
-  <si>
-    <t>AN/2854/2026</t>
-  </si>
-  <si>
-    <t>AN/2855/2026</t>
-  </si>
-  <si>
-    <t>AN/2856/2026</t>
-  </si>
-  <si>
-    <t>AN/2857/2026</t>
-  </si>
-  <si>
-    <t>AN/2858/2026</t>
-  </si>
-  <si>
-    <t>AN/2859/2026</t>
-  </si>
-  <si>
-    <t>AN/2860/2026</t>
-  </si>
-  <si>
-    <t>AN/2961/2026</t>
-  </si>
-  <si>
-    <t>17-06-26</t>
-  </si>
-  <si>
-    <t>15</t>
+    <t>JOSE ANGEL SAMANIEGO</t>
+  </si>
+  <si>
+    <t>FI26-1C046A327-2B8C-4F66-9382-70E1D52B8DC9</t>
+  </si>
+  <si>
+    <t>ALISON AISLINN DE SANTIAGO RAMIREZ</t>
+  </si>
+  <si>
+    <t>FI26-13A42ACC2-15E1-4FAE-9441-E77DA227C8AA</t>
+  </si>
+  <si>
+    <t>QUERETARO</t>
+  </si>
+  <si>
+    <t>FISCALIA GENERAL DEL ESTADO QUERETARO</t>
+  </si>
+  <si>
+    <t>RODIBERTO DE LA FLOR ARGUELLEZ</t>
+  </si>
+  <si>
+    <t>FI26-1F0F5F526-ACCA-4544-A330-4400068F1D5B</t>
+  </si>
+  <si>
+    <t>CHIAPAS</t>
+  </si>
+  <si>
+    <t>FISCALIA GENERAL DEL ESTADO DE CHIAPAS</t>
+  </si>
+  <si>
+    <t>OLIVER JOSUE RODRIGUEZ RUIZ</t>
+  </si>
+  <si>
+    <t>FI26-103D2F719-ECDD-4E59-93DB-9B6A02AFE3FB</t>
+  </si>
+  <si>
+    <t>CAMISA, PANTALÓN COLOR: AZUL MARINO, 
+TENIS COLOR: NEGRO/BLANCO</t>
+  </si>
+  <si>
+    <t>COMPLEXION: MEDIANACARA: OVALADOCOLOR DE LA PIEL: BLANCOCABELLO:
+ CASTAÑO OSCURO CORTO LISOOJOS: CAFÉS MEDIANOSNARIZ: RECTABOCA:
+ GRANDELABIOS: DELGADOSESTATURA: 190 CMPESO: 
+110KG CUENTA CON VARIOS TATUAJES, ENTRE ELLOS UNA CARA DEL DIABLO, 
+CALAVERAS, UNA CRUZ AMBER RENATA,</t>
   </si>
 </sst>
 </file>
@@ -243,7 +417,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -265,6 +439,9 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -616,8 +793,8 @@
     <col min="13" max="13" width="21.5546875" style="5" customWidth="1"/>
     <col min="14" max="14" width="58.6640625" style="5" customWidth="1"/>
     <col min="15" max="15" width="16.33203125" style="5" customWidth="1"/>
-    <col min="16" max="23" width="11.5546875" style="5" customWidth="1"/>
-    <col min="24" max="16384" width="11.5546875" style="5"/>
+    <col min="16" max="25" width="11.5546875" style="5" customWidth="1"/>
+    <col min="26" max="16384" width="11.5546875" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="1" customFormat="1" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -669,13 +846,13 @@
         <v>2846</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E2" s="5">
         <v>15</v>
@@ -684,28 +861,28 @@
         <v>15</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -713,7 +890,43 @@
         <v>2847</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>24</v>
+        <v>35</v>
+      </c>
+      <c r="C3" s="10">
+        <v>46199</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3" s="5">
+        <v>56</v>
+      </c>
+      <c r="F3" s="5">
+        <v>56</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="K3" s="8">
+        <v>46183</v>
+      </c>
+      <c r="L3" s="10">
+        <v>46184</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -721,7 +934,43 @@
         <v>2848</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>26</v>
+        <v>50</v>
+      </c>
+      <c r="C4" s="10">
+        <v>46199</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="5">
+        <v>21</v>
+      </c>
+      <c r="F4" s="5">
+        <v>21</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="K4" s="8">
+        <v>46093</v>
+      </c>
+      <c r="L4" s="10">
+        <v>46192</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -729,7 +978,43 @@
         <v>2849</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
+      </c>
+      <c r="C5" s="10">
+        <v>46199</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5" s="5">
+        <v>43</v>
+      </c>
+      <c r="F5" s="5">
+        <v>43</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="K5" s="8">
+        <v>46192</v>
+      </c>
+      <c r="L5" s="10">
+        <v>46192</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -737,7 +1022,43 @@
         <v>2850</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>28</v>
+        <v>69</v>
+      </c>
+      <c r="C6" s="10">
+        <v>46199</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" s="5">
+        <v>21</v>
+      </c>
+      <c r="F6" s="5">
+        <v>22</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="K6" s="8">
+        <v>46088</v>
+      </c>
+      <c r="L6" s="10">
+        <v>46088</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -745,7 +1066,43 @@
         <v>2851</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>29</v>
+        <v>70</v>
+      </c>
+      <c r="C7" s="10">
+        <v>46199</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="5">
+        <v>36</v>
+      </c>
+      <c r="F7" s="5">
+        <v>36</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K7" s="8">
+        <v>46086</v>
+      </c>
+      <c r="L7" s="10">
+        <v>46086</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -753,7 +1110,43 @@
         <v>2852</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="10">
+        <v>46199</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="5">
+        <v>45</v>
+      </c>
+      <c r="F8" s="5">
+        <v>45</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" s="5" t="s">
         <v>30</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K8" s="8">
+        <v>46172</v>
+      </c>
+      <c r="L8" s="10">
+        <v>46172</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -761,17 +1154,51 @@
         <v>2853</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="10"/>
-      <c r="L9" s="10"/>
+        <v>72</v>
+      </c>
+      <c r="C9" s="10">
+        <v>46199</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="5">
+        <v>6</v>
+      </c>
+      <c r="F9" s="5">
+        <v>6</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="K9" s="8">
+        <v>46192</v>
+      </c>
+      <c r="L9" s="10">
+        <v>46192</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>2854</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="C10" s="10"/>
       <c r="L10" s="10"/>
@@ -781,7 +1208,7 @@
         <v>2855</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="C11" s="10"/>
       <c r="L11" s="10"/>
@@ -791,7 +1218,7 @@
         <v>2856</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="C12" s="10"/>
       <c r="L12" s="10"/>
@@ -801,7 +1228,7 @@
         <v>2857</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -809,7 +1236,7 @@
         <v>2858</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>36</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -817,7 +1244,7 @@
         <v>2859</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>37</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -825,7 +1252,7 @@
         <v>2860</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>38</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
@@ -1333,43 +1760,1072 @@
         <v>2961</v>
       </c>
       <c r="B117" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C117" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D117" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E117" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F117" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G117" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H117" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I117" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="J117" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K117" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="L117" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M117" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="N117" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:Y117"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.5546875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="17.44140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="16.109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="36.88671875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" style="5" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" style="5" customWidth="1"/>
+    <col min="7" max="8" width="11.5546875" style="5" customWidth="1"/>
+    <col min="9" max="9" width="15.33203125" style="5" customWidth="1"/>
+    <col min="10" max="10" width="44.109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="14.88671875" style="8" customWidth="1"/>
+    <col min="12" max="12" width="15.44140625" style="5" customWidth="1"/>
+    <col min="13" max="13" width="21.5546875" style="5" customWidth="1"/>
+    <col min="14" max="14" width="58.6640625" style="5" customWidth="1"/>
+    <col min="15" max="15" width="16.33203125" style="5" customWidth="1"/>
+    <col min="16" max="16" width="26.5546875" style="5" customWidth="1"/>
+    <col min="17" max="17" width="15.88671875" style="5" customWidth="1"/>
+    <col min="18" max="18" width="18" style="5" customWidth="1"/>
+    <col min="19" max="19" width="16.88671875" style="5" customWidth="1"/>
+    <col min="20" max="20" width="38.5546875" style="5" customWidth="1"/>
+    <col min="21" max="21" width="31.88671875" style="5" customWidth="1"/>
+    <col min="22" max="22" width="74.33203125" style="5" customWidth="1"/>
+    <col min="23" max="23" width="48.77734375" style="5" customWidth="1"/>
+    <col min="24" max="24" width="38.109375" style="5" customWidth="1"/>
+    <col min="25" max="25" width="26.88671875" style="5" customWidth="1"/>
+    <col min="26" max="26" width="20.6640625" style="5" customWidth="1"/>
+    <col min="27" max="27" width="11.5546875" style="5" customWidth="1"/>
+    <col min="28" max="16384" width="11.5546875" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:25" s="1" customFormat="1" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>2846</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="5">
+        <v>15</v>
+      </c>
+      <c r="F2" s="5">
+        <v>15</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>2847</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="10">
+        <v>46205</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="5">
+        <v>36</v>
+      </c>
+      <c r="F3" s="5">
+        <v>36</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J3" s="5" t="s">
         <v>39</v>
       </c>
+      <c r="K3" s="8">
+        <v>46086</v>
+      </c>
+      <c r="L3" s="10">
+        <v>46086</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="V3" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="X3" s="11" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>2848</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="10">
+        <v>46205</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="5">
+        <v>45</v>
+      </c>
+      <c r="F4" s="5">
+        <v>45</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K4" s="8">
+        <v>46172</v>
+      </c>
+      <c r="L4" s="10">
+        <v>46172</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="T4" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>2849</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="10">
+        <v>46205</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E5" s="5">
+        <v>6</v>
+      </c>
+      <c r="F5" s="5">
+        <v>6</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="K5" s="8">
+        <v>46192</v>
+      </c>
+      <c r="L5" s="10">
+        <v>46192</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="X5" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>2850</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="10"/>
+      <c r="L6" s="10"/>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>2851</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="10"/>
+      <c r="L7" s="10"/>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>2852</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="L8" s="10"/>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>2853</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" s="10"/>
+      <c r="L9" s="10"/>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>2854</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="10"/>
+      <c r="L10" s="10"/>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>2855</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="10"/>
+      <c r="L11" s="10"/>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
+        <v>2856</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" s="10"/>
+      <c r="L12" s="10"/>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
+        <v>2857</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
+        <v>2858</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
+        <v>2859</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
+        <v>2860</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
+        <v>2861</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
+        <v>2862</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
+        <v>2863</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
+        <v>2864</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
+        <v>2865</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
+        <v>2866</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
+        <v>2867</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
+        <v>2868</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
+        <v>2869</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
+        <v>2870</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
+        <v>2871</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
+        <v>2872</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
+        <v>2873</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
+        <v>2874</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
+        <v>2875</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
+        <v>2876</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
+        <v>2877</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" s="3">
+        <v>2878</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" s="3">
+        <v>2879</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
+        <v>2880</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
+        <v>2881</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
+        <v>2882</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39" s="3">
+        <v>2883</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40" s="3">
+        <v>2884</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41" s="3">
+        <v>2885</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A42" s="3">
+        <v>2886</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43" s="3">
+        <v>2887</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44" s="3">
+        <v>2888</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A45" s="3">
+        <v>2889</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A46" s="3">
+        <v>2890</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47" s="3">
+        <v>2891</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48" s="3">
+        <v>2892</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" s="3">
+        <v>2893</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="3">
+        <v>2894</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" s="3">
+        <v>2895</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" s="3">
+        <v>2896</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" s="3">
+        <v>2897</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54" s="3">
+        <v>2898</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" s="3">
+        <v>2899</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" s="3">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" s="3">
+        <v>2901</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" s="3">
+        <v>2902</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" s="3">
+        <v>2903</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" s="3">
+        <v>2904</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A61" s="3">
+        <v>2905</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A62" s="3">
+        <v>2906</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" s="3">
+        <v>2907</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A64" s="3">
+        <v>2908</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A65" s="3">
+        <v>2909</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A66" s="3">
+        <v>2910</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A67" s="3">
+        <v>2911</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A68" s="3">
+        <v>2912</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A69" s="3">
+        <v>2913</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A70" s="3">
+        <v>2914</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A71" s="3">
+        <v>2915</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A72" s="3">
+        <v>2916</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A73" s="3">
+        <v>2917</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A74" s="3">
+        <v>2918</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A75" s="3">
+        <v>2919</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A76" s="3">
+        <v>2920</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A77" s="3">
+        <v>2921</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A78" s="3">
+        <v>2922</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A79" s="3">
+        <v>2923</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A80" s="3">
+        <v>2924</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A81" s="3">
+        <v>2925</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A82" s="3">
+        <v>2926</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A83" s="3">
+        <v>2927</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A84" s="3">
+        <v>2928</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A85" s="3">
+        <v>2929</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A86" s="3">
+        <v>2930</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A87" s="3">
+        <v>2931</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A88" s="3">
+        <v>2932</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A89" s="3">
+        <v>2933</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A90" s="3">
+        <v>2934</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A91" s="3">
+        <v>2935</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A92" s="3">
+        <v>2936</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A93" s="3">
+        <v>2937</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A94" s="3">
+        <v>2938</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A95" s="3">
+        <v>2939</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A96" s="3">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A97" s="3">
+        <v>2941</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A98" s="3">
+        <v>2942</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A99" s="3">
+        <v>2943</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A100" s="3">
+        <v>2944</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A101" s="3">
+        <v>2945</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A102" s="3">
+        <v>2946</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A103" s="3">
+        <v>2947</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A104" s="3">
+        <v>2948</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A105" s="3">
+        <v>2949</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A106" s="3">
+        <v>2950</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A107" s="3">
+        <v>2951</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A108" s="3">
+        <v>2952</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A109" s="3">
+        <v>2953</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A110" s="3">
+        <v>2954</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A111" s="3">
+        <v>2955</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A112" s="3">
+        <v>2956</v>
+      </c>
+    </row>
+    <row r="113" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A113" s="3">
+        <v>2957</v>
+      </c>
+    </row>
+    <row r="114" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A114" s="3">
+        <v>2958</v>
+      </c>
+    </row>
+    <row r="115" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A115" s="3">
+        <v>2959</v>
+      </c>
+    </row>
+    <row r="116" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A116" s="3">
+        <v>2960</v>
+      </c>
+    </row>
+    <row r="117" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A117" s="6">
+        <v>2961</v>
+      </c>
+      <c r="B117" s="6" t="s">
+        <v>80</v>
+      </c>
       <c r="C117" s="6" t="s">
-        <v>40</v>
+        <v>81</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>41</v>
+        <v>82</v>
       </c>
       <c r="F117" s="6" t="s">
-        <v>41</v>
+        <v>82</v>
       </c>
       <c r="G117" s="6" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H117" s="6" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="I117" s="6" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="J117" s="6" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="K117" s="9" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="L117" s="6" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="M117" s="6" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="N117" s="6" t="s">
-        <v>25</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>